<commit_message>
code update for result details row
</commit_message>
<xml_diff>
--- a/Rules.xlsx
+++ b/Rules.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="67">
   <si>
     <t xml:space="preserve">Rule No </t>
   </si>
@@ -426,6 +426,15 @@
   </si>
   <si>
     <t>Total Cost</t>
+  </si>
+  <si>
+    <t>R8.1</t>
+  </si>
+  <si>
+    <t>(∑&lt;Monthly ZeroProfit Premium&gt;,&lt;Monthly Claim Cost&gt;,&lt;Monthly FullProfit Premium&gt;,&lt;Monthly Base Claim Cost&gt;) x 12</t>
+  </si>
+  <si>
+    <t>Annual Total Cost</t>
   </si>
 </sst>
 </file>
@@ -1020,7 +1029,20 @@
         <v>63</v>
       </c>
     </row>
-    <row r="22" ht="14.25" customHeight="1"/>
+    <row r="22" ht="14.25" customHeight="1">
+      <c r="A22" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
     <row r="23" ht="14.25" customHeight="1"/>
     <row r="24" ht="14.25" customHeight="1"/>
     <row r="25" ht="14.25" customHeight="1"/>

</xml_diff>